<commit_message>
Flatten source layout and preserve package imports
</commit_message>
<xml_diff>
--- a/docs/providers/源头采集接口说明.xlsx
+++ b/docs/providers/源头采集接口说明.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总览" sheetId="1" r:id="R8aec7a0f1a614729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用参数" sheetId="2" r:id="R6e4de46436e14036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集字段与映射" sheetId="3" r:id="R649a9085437e47ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="暂不纳入及历史" sheetId="4" r:id="Rf83c3583e42c48cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总览" sheetId="1" r:id="Rca9353452b4e499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用参数" sheetId="2" r:id="Rfc05784fa9b04ee5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集字段与映射" sheetId="3" r:id="R7d0c5e5cf1e747ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="暂不纳入及历史" sheetId="4" r:id="R770a3fd42a414035"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -533,7 +533,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.56727313658</x:v>
+        <x:v>46299.680338136575</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -926,7 +926,7 @@
       </x:c>
       <x:c r="AD10" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-001
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -1023,7 +1023,7 @@
       </x:c>
       <x:c r="AD11" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-002-5m
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -1116,7 +1116,7 @@
       </x:c>
       <x:c r="AD12" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-002-daily
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="89" customHeight="1">
@@ -1216,7 +1216,7 @@
       </x:c>
       <x:c r="AD13" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-003
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="89" customHeight="1">
@@ -1317,7 +1317,7 @@
       </x:c>
       <x:c r="AD14" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-004
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">
@@ -1414,7 +1414,7 @@
       </x:c>
       <x:c r="AD15" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-006
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="103" customHeight="1">
@@ -1512,7 +1512,7 @@
       </x:c>
       <x:c r="AD16" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-008
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="76" customHeight="1">
@@ -1609,7 +1609,7 @@
       </x:c>
       <x:c r="AD17" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-013
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="1075" customHeight="1">
@@ -1748,7 +1748,7 @@
       </x:c>
       <x:c r="AD18" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-014
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="116" customHeight="1">
@@ -1847,7 +1847,7 @@
       </x:c>
       <x:c r="AD19" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-019
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="116" customHeight="1">
@@ -1947,7 +1947,7 @@
       </x:c>
       <x:c r="AD20" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-020
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="103" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="AD21" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-021
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="89" customHeight="1">
@@ -2143,7 +2143,7 @@
       </x:c>
       <x:c r="AD22" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-026
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="89" customHeight="1">
@@ -2242,7 +2242,7 @@
       </x:c>
       <x:c r="AD23" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-027
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="89" customHeight="1">
@@ -2341,7 +2341,7 @@
       </x:c>
       <x:c r="AD24" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-028
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="89" customHeight="1">
@@ -2442,7 +2442,7 @@
       </x:c>
       <x:c r="AD25" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-030
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="89" customHeight="1">
@@ -2543,7 +2543,7 @@
       </x:c>
       <x:c r="AD26" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-031
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="89" customHeight="1">
@@ -2641,7 +2641,7 @@
       </x:c>
       <x:c r="AD27" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-032
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="89" customHeight="1">
@@ -2740,7 +2740,7 @@
       </x:c>
       <x:c r="AD28" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-033
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="89" customHeight="1">
@@ -2838,7 +2838,7 @@
       </x:c>
       <x:c r="AD29" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-034
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="89" customHeight="1">
@@ -2936,7 +2936,7 @@
       </x:c>
       <x:c r="AD30" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-035
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="89" customHeight="1">
@@ -3037,7 +3037,7 @@
       </x:c>
       <x:c r="AD31" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-039
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="103" customHeight="1">
@@ -3137,7 +3137,7 @@
       </x:c>
       <x:c r="AD32" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-044
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="89" customHeight="1">
@@ -3229,7 +3229,7 @@
       </x:c>
       <x:c r="AD33" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-045
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="89" customHeight="1">
@@ -3327,7 +3327,7 @@
       </x:c>
       <x:c r="AD34" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-046
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="89" customHeight="1">
@@ -3425,7 +3425,7 @@
       </x:c>
       <x:c r="AD35" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-047
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="89" customHeight="1">
@@ -3523,7 +3523,7 @@
       </x:c>
       <x:c r="AD36" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-048
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="89" customHeight="1">
@@ -3622,7 +3622,7 @@
       </x:c>
       <x:c r="AD37" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-050
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="89" customHeight="1">
@@ -3723,7 +3723,7 @@
       </x:c>
       <x:c r="AD38" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-051
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="89" customHeight="1">
@@ -3824,7 +3824,7 @@
       </x:c>
       <x:c r="AD39" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-055
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="116" customHeight="1">
@@ -3923,7 +3923,7 @@
       </x:c>
       <x:c r="AD40" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-061
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="89" customHeight="1">
@@ -4021,7 +4021,7 @@
       </x:c>
       <x:c r="AD41" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-062
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="76" customHeight="1">
@@ -4120,7 +4120,7 @@
       </x:c>
       <x:c r="AD42" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-063
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="103" customHeight="1">
@@ -4222,7 +4222,7 @@
       </x:c>
       <x:c r="AD43" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-064
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="89" customHeight="1">
@@ -4323,7 +4323,7 @@
       </x:c>
       <x:c r="AD44" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-065
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="76" customHeight="1">
@@ -4418,7 +4418,7 @@
       </x:c>
       <x:c r="AD45" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-066
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="103" customHeight="1">
@@ -4519,7 +4519,7 @@
       </x:c>
       <x:c r="AD46" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-067
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="103" customHeight="1">
@@ -4620,7 +4620,7 @@
       </x:c>
       <x:c r="AD47" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-068
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="103" customHeight="1">
@@ -4723,7 +4723,7 @@
       </x:c>
       <x:c r="AD48" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-069
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="89" customHeight="1">
@@ -4816,7 +4816,7 @@
       </x:c>
       <x:c r="AD49" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-070
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="103" customHeight="1">
@@ -4918,7 +4918,7 @@
       </x:c>
       <x:c r="AD50" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-071
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="103" customHeight="1">
@@ -5021,7 +5021,7 @@
       </x:c>
       <x:c r="AD51" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-072
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="116" customHeight="1">
@@ -5129,7 +5129,7 @@
       </x:c>
       <x:c r="AD52" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-073
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="103" customHeight="1">
@@ -5231,7 +5231,7 @@
       </x:c>
       <x:c r="AD53" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-074
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="103" customHeight="1">
@@ -5331,7 +5331,7 @@
       </x:c>
       <x:c r="AD54" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-075
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="103" customHeight="1">
@@ -5433,7 +5433,7 @@
       </x:c>
       <x:c r="AD55" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-076
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="103" customHeight="1">
@@ -5534,7 +5534,7 @@
       </x:c>
       <x:c r="AD56" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-077
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="89" customHeight="1">
@@ -5634,7 +5634,7 @@
       </x:c>
       <x:c r="AD57" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-078
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="89" customHeight="1">
@@ -5732,7 +5732,7 @@
       </x:c>
       <x:c r="AD58" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-079
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="89" customHeight="1">
@@ -5832,7 +5832,7 @@
       </x:c>
       <x:c r="AD59" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-080
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="89" customHeight="1">
@@ -5933,7 +5933,7 @@
       </x:c>
       <x:c r="AD60" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-081
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="103" customHeight="1">
@@ -6035,7 +6035,7 @@
       </x:c>
       <x:c r="AD61" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-082
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="89" customHeight="1">
@@ -6136,7 +6136,7 @@
       </x:c>
       <x:c r="AD62" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-083
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="116" customHeight="1">
@@ -6239,7 +6239,7 @@
       </x:c>
       <x:c r="AD63" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-084
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="89" customHeight="1">
@@ -6339,7 +6339,7 @@
       </x:c>
       <x:c r="AD64" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-085
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="103" customHeight="1">
@@ -6439,7 +6439,7 @@
       </x:c>
       <x:c r="AD65" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-087
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="62" customHeight="1">
@@ -6532,7 +6532,7 @@
       </x:c>
       <x:c r="AD66" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-001
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="62" customHeight="1">
@@ -6626,7 +6626,7 @@
       </x:c>
       <x:c r="AD67" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-002
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="89" customHeight="1">
@@ -6721,7 +6721,7 @@
       </x:c>
       <x:c r="AD68" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-003
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="251" customHeight="1">
@@ -6822,7 +6822,7 @@
       </x:c>
       <x:c r="AD69" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-004
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="89" customHeight="1">
@@ -6917,7 +6917,7 @@
       </x:c>
       <x:c r="AD70" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-005
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="76" customHeight="1">
@@ -7012,7 +7012,7 @@
       </x:c>
       <x:c r="AD71" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-006
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="89" customHeight="1">
@@ -7111,7 +7111,7 @@
       </x:c>
       <x:c r="AD72" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-037-profile
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="103" customHeight="1">
@@ -7211,13 +7211,13 @@
       </x:c>
       <x:c r="AD73" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-037-events
-src/stock_data_manage/routing/factory.py</x:v>
+src/routing/factory.py</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6bf1888beaa4284"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d69ae4881b4b29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7287,7 +7287,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.56727313658</x:v>
+        <x:v>46299.680338136575</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -12398,7 +12398,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd836555f73ba4dd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4702f5b6e1b44f90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12477,7 +12477,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.56727313658</x:v>
+        <x:v>46299.680338136575</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -68968,7 +68968,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c03758786ec4b5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R048dd8b2f1d747db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -69020,7 +69020,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.56727313658</x:v>
+        <x:v>46299.680338136575</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -69478,7 +69478,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc65d075550e34d5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2593b588e498429c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Unify runtime storage layers and guard task archival
</commit_message>
<xml_diff>
--- a/docs/providers/源头采集接口说明.xlsx
+++ b/docs/providers/源头采集接口说明.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总览" sheetId="1" r:id="Rca9353452b4e499b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用参数" sheetId="2" r:id="Rfc05784fa9b04ee5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集字段与映射" sheetId="3" r:id="R7d0c5e5cf1e747ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="暂不纳入及历史" sheetId="4" r:id="R770a3fd42a414035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="接口总览" sheetId="1" r:id="Rc27433d7382a4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用参数" sheetId="2" r:id="R97a6026011be422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集字段与映射" sheetId="3" r:id="R0d2b54ad53b74028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="暂不纳入及历史" sheetId="4" r:id="R7e018baaa3ba4e56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -125,9 +125,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FormalProviderSpec0" displayName="FormalProviderSpec0" ref="A9:AD73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A9:AD73"/>
-  <x:tableColumns count="30">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FormalProviderSpec0" displayName="FormalProviderSpec0" ref="A9:AI73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A9:AI73"/>
+  <x:tableColumns count="35">
     <x:tableColumn id="1" name="输入ID"/>
     <x:tableColumn id="2" name="能力名称"/>
     <x:tableColumn id="3" name="来源"/>
@@ -158,6 +158,11 @@
     <x:tableColumn id="28" name="验证报告"/>
     <x:tableColumn id="29" name="原始证据清单"/>
     <x:tableColumn id="30" name="配置与代码入口"/>
+    <x:tableColumn id="31" name="运行原始响应路径"/>
+    <x:tableColumn id="32" name="任务工作区路径"/>
+    <x:tableColumn id="33" name="来源标准化文件"/>
+    <x:tableColumn id="34" name="最终数据与发布状态"/>
+    <x:tableColumn id="35" name="任务归档条件"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -460,6 +465,11 @@
     <x:col min="28" max="28" width="55" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="55" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="55" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="55" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="55" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="55" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="55" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -493,6 +503,11 @@
       <x:c r="AB1" s="2"/>
       <x:c r="AC1" s="2"/>
       <x:c r="AD1" s="2"/>
+      <x:c r="AE1" s="2"/>
+      <x:c r="AF1" s="2"/>
+      <x:c r="AG1" s="2"/>
+      <x:c r="AH1" s="2"/>
+      <x:c r="AI1" s="2"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -527,13 +542,18 @@
       <x:c r="AB2" s="2"/>
       <x:c r="AC2" s="2"/>
       <x:c r="AD2" s="2"/>
+      <x:c r="AE2" s="2"/>
+      <x:c r="AF2" s="2"/>
+      <x:c r="AG2" s="2"/>
+      <x:c r="AH2" s="2"/>
+      <x:c r="AI2" s="2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.680338136575</x:v>
+        <x:v>46299.7938500463</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -563,6 +583,11 @@
       <x:c r="AB3" s="2"/>
       <x:c r="AC3" s="2"/>
       <x:c r="AD3" s="2"/>
+      <x:c r="AE3" s="2"/>
+      <x:c r="AF3" s="2"/>
+      <x:c r="AG3" s="2"/>
+      <x:c r="AH3" s="2"/>
+      <x:c r="AI3" s="2"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="2" t="str">
@@ -605,6 +630,11 @@
       <x:c r="AB4" s="2"/>
       <x:c r="AC4" s="2"/>
       <x:c r="AD4" s="2"/>
+      <x:c r="AE4" s="2"/>
+      <x:c r="AF4" s="2"/>
+      <x:c r="AG4" s="2"/>
+      <x:c r="AH4" s="2"/>
+      <x:c r="AI4" s="2"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="2"/>
@@ -637,6 +667,11 @@
       <x:c r="AB5" s="2"/>
       <x:c r="AC5" s="2"/>
       <x:c r="AD5" s="2"/>
+      <x:c r="AE5" s="2"/>
+      <x:c r="AF5" s="2"/>
+      <x:c r="AG5" s="2"/>
+      <x:c r="AH5" s="2"/>
+      <x:c r="AI5" s="2"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="5" t="str">
@@ -671,6 +706,11 @@
       <x:c r="AB6" s="2"/>
       <x:c r="AC6" s="2"/>
       <x:c r="AD6" s="2"/>
+      <x:c r="AE6" s="2"/>
+      <x:c r="AF6" s="2"/>
+      <x:c r="AG6" s="2"/>
+      <x:c r="AH6" s="2"/>
+      <x:c r="AI6" s="2"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="5" t="str">
@@ -705,6 +745,11 @@
       <x:c r="AB7" s="2"/>
       <x:c r="AC7" s="2"/>
       <x:c r="AD7" s="2"/>
+      <x:c r="AE7" s="2"/>
+      <x:c r="AF7" s="2"/>
+      <x:c r="AG7" s="2"/>
+      <x:c r="AH7" s="2"/>
+      <x:c r="AI7" s="2"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="2"/>
@@ -737,6 +782,11 @@
       <x:c r="AB8" s="2"/>
       <x:c r="AC8" s="2"/>
       <x:c r="AD8" s="2"/>
+      <x:c r="AE8" s="2"/>
+      <x:c r="AF8" s="2"/>
+      <x:c r="AG8" s="2"/>
+      <x:c r="AH8" s="2"/>
+      <x:c r="AI8" s="2"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="9" t="str">
@@ -828,6 +878,21 @@
       </x:c>
       <x:c r="AD9" s="9" t="str">
         <x:v>配置与代码入口</x:v>
+      </x:c>
+      <x:c r="AE9" s="9" t="str">
+        <x:v>运行原始响应路径</x:v>
+      </x:c>
+      <x:c r="AF9" s="9" t="str">
+        <x:v>任务工作区路径</x:v>
+      </x:c>
+      <x:c r="AG9" s="9" t="str">
+        <x:v>来源标准化文件</x:v>
+      </x:c>
+      <x:c r="AH9" s="9" t="str">
+        <x:v>最终数据与发布状态</x:v>
+      </x:c>
+      <x:c r="AI9" s="9" t="str">
+        <x:v>任务归档条件</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="89" customHeight="1">
@@ -928,6 +993,25 @@
         <x:v>config/providers.yaml#ASTOCK-001
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE10" s="6" t="str">
+        <x:v>data/raw/tencent/single_quote/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF10" s="6" t="str">
+        <x:v>data/task_workspace/realtime_quote/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG10" s="6" t="str">
+        <x:v>sources/tencent/ASTOCK-001/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH10" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI10" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -1025,6 +1109,25 @@
         <x:v>config/providers.yaml#ASTOCK-002-5m
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE11" s="6" t="str">
+        <x:v>data/raw/tencent/kline_5m/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF11" s="6" t="str">
+        <x:v>data/task_workspace/minute_bar_5m/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG11" s="6" t="str">
+        <x:v>sources/tencent/ASTOCK-002-5m/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH11" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI11" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -1117,6 +1220,25 @@
       <x:c r="AD12" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-002-daily
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE12" s="6" t="str">
+        <x:v>data/raw/tencent/kline_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF12" s="6" t="str">
+        <x:v>data/task_workspace/daily_bar/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG12" s="6" t="str">
+        <x:v>sources/tencent/ASTOCK-002-daily/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH12" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI12" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="89" customHeight="1">
@@ -1218,6 +1340,25 @@
         <x:v>config/providers.yaml#ASTOCK-003
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE13" s="6" t="str">
+        <x:v>data/raw/tdx/daily_package/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF13" s="6" t="str">
+        <x:v>data/task_workspace/tdx_daily_package/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG13" s="6" t="str">
+        <x:v>sources/tdx/ASTOCK-003/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH13" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI13" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="89" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -1319,6 +1460,25 @@
         <x:v>config/providers.yaml#ASTOCK-004
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE14" s="6" t="str">
+        <x:v>data/raw/tencent/ticks/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF14" s="6" t="str">
+        <x:v>data/task_workspace/tencent_ticks/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG14" s="6" t="str">
+        <x:v>sources/tencent/ASTOCK-004/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH14" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI14" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -1415,6 +1575,25 @@
       <x:c r="AD15" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-006
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE15" s="6" t="str">
+        <x:v>data/raw/sina/adjustment_factor/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF15" s="6" t="str">
+        <x:v>data/task_workspace/adjustment_factor/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG15" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-006/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH15" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI15" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="103" customHeight="1">
@@ -1514,6 +1693,25 @@
         <x:v>config/providers.yaml#ASTOCK-008
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE16" s="6" t="str">
+        <x:v>data/raw/eastmoney/report_list/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF16" s="6" t="str">
+        <x:v>data/task_workspace/eastmoney_reports/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG16" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-008/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH16" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI16" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="76" customHeight="1">
       <x:c r="A17" s="12" t="str">
@@ -1610,6 +1808,25 @@
       <x:c r="AD17" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-013
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE17" s="6" t="str">
+        <x:v>data/raw/sina/report_list/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF17" s="6" t="str">
+        <x:v>data/task_workspace/sina_reports/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG17" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-013/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH17" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI17" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="1075" customHeight="1">
@@ -1750,6 +1967,25 @@
         <x:v>config/providers.yaml#ASTOCK-014
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE18" s="6" t="str">
+        <x:v>data/raw/ths/concept_directory/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF18" s="6" t="str">
+        <x:v>data/task_workspace/concept_directory/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG18" s="6" t="str">
+        <x:v>sources/ths/ASTOCK-014/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH18" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI18" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="116" customHeight="1">
       <x:c r="A19" s="12" t="str">
@@ -1849,6 +2085,25 @@
         <x:v>config/providers.yaml#ASTOCK-019
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE19" s="6" t="str">
+        <x:v>data/raw/eastmoney/dragon_tiger_seats/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF19" s="6" t="str">
+        <x:v>data/task_workspace/dragon_tiger_seats/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG19" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-019/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH19" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI19" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="116" customHeight="1">
       <x:c r="A20" s="12" t="str">
@@ -1949,6 +2204,25 @@
         <x:v>config/providers.yaml#ASTOCK-020
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE20" s="6" t="str">
+        <x:v>data/raw/eastmoney/dragon_tiger_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF20" s="6" t="str">
+        <x:v>data/task_workspace/dragon_tiger_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG20" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-020/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH20" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI20" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="103" customHeight="1">
       <x:c r="A21" s="12" t="str">
@@ -2046,6 +2320,25 @@
       <x:c r="AD21" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-021
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE21" s="6" t="str">
+        <x:v>data/raw/eastmoney/lockup_expiry/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF21" s="6" t="str">
+        <x:v>data/task_workspace/lockup_expiry/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG21" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-021/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH21" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI21" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="89" customHeight="1">
@@ -2145,6 +2438,25 @@
         <x:v>config/providers.yaml#ASTOCK-026
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE22" s="6" t="str">
+        <x:v>data/raw/eastmoney/shareholder_count/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF22" s="6" t="str">
+        <x:v>data/task_workspace/shareholder_count/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG22" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-026/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH22" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI22" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="89" customHeight="1">
       <x:c r="A23" s="12" t="str">
@@ -2244,6 +2556,25 @@
         <x:v>config/providers.yaml#ASTOCK-027
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE23" s="6" t="str">
+        <x:v>data/raw/eastmoney/dividend_history/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF23" s="6" t="str">
+        <x:v>data/task_workspace/dividend_event/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG23" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-027/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH23" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI23" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="89" customHeight="1">
       <x:c r="A24" s="12" t="str">
@@ -2342,6 +2673,25 @@
       <x:c r="AD24" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-028
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE24" s="6" t="str">
+        <x:v>data/raw/eastmoney/stock_fund_flow/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF24" s="6" t="str">
+        <x:v>data/task_workspace/stock_fund_flow/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG24" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-028/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH24" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI24" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="89" customHeight="1">
@@ -2444,6 +2794,25 @@
         <x:v>config/providers.yaml#ASTOCK-030
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE25" s="6" t="str">
+        <x:v>data/raw/sse/etf_shares/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF25" s="6" t="str">
+        <x:v>data/task_workspace/etf_shares/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG25" s="6" t="str">
+        <x:v>sources/sse/ASTOCK-030/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH25" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI25" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="89" customHeight="1">
       <x:c r="A26" s="12" t="str">
@@ -2545,6 +2914,25 @@
         <x:v>config/providers.yaml#ASTOCK-031
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE26" s="6" t="str">
+        <x:v>data/raw/eastmoney/stock_news/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF26" s="6" t="str">
+        <x:v>data/task_workspace/stock_news/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG26" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-031/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH26" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI26" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="89" customHeight="1">
       <x:c r="A27" s="12" t="str">
@@ -2643,6 +3031,25 @@
         <x:v>config/providers.yaml#ASTOCK-032
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE27" s="6" t="str">
+        <x:v>data/raw/cls/telegraph/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF27" s="6" t="str">
+        <x:v>data/task_workspace/cls_telegraph/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG27" s="6" t="str">
+        <x:v>sources/cls/ASTOCK-032/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH27" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI27" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="89" customHeight="1">
       <x:c r="A28" s="12" t="str">
@@ -2742,6 +3149,25 @@
         <x:v>config/providers.yaml#ASTOCK-033
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE28" s="6" t="str">
+        <x:v>data/raw/sina/global_news/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF28" s="6" t="str">
+        <x:v>data/task_workspace/sina_global_news/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG28" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-033/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH28" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI28" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="89" customHeight="1">
       <x:c r="A29" s="12" t="str">
@@ -2840,6 +3266,25 @@
         <x:v>config/providers.yaml#ASTOCK-034
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE29" s="6" t="str">
+        <x:v>data/raw/wallstreetcn/news_lives/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF29" s="6" t="str">
+        <x:v>data/task_workspace/wallstreetcn_news/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG29" s="6" t="str">
+        <x:v>sources/wallstreetcn/ASTOCK-034/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH29" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI29" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="89" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -2937,6 +3382,25 @@
       <x:c r="AD30" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-035
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE30" s="6" t="str">
+        <x:v>data/raw/cctv/news/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF30" s="6" t="str">
+        <x:v>data/task_workspace/cctv_news_index/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG30" s="6" t="str">
+        <x:v>sources/cctv/ASTOCK-035/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH30" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI30" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="89" customHeight="1">
@@ -3038,6 +3502,25 @@
       <x:c r="AD31" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-039
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE31" s="6" t="str">
+        <x:v>data/raw/sina/financial_statements/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF31" s="6" t="str">
+        <x:v>data/task_workspace/sina_financial_statements/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG31" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-039/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH31" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI31" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="103" customHeight="1">
@@ -3139,6 +3622,25 @@
         <x:v>config/providers.yaml#ASTOCK-044
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE32" s="6" t="str">
+        <x:v>data/raw/baostock/st_list/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF32" s="6" t="str">
+        <x:v>data/task_workspace/st_name_list/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG32" s="6" t="str">
+        <x:v>sources/baostock/ASTOCK-044/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH32" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI32" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="89" customHeight="1">
       <x:c r="A33" s="12" t="str">
@@ -3230,6 +3732,25 @@
       <x:c r="AD33" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-045
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE33" s="6" t="str">
+        <x:v>data/raw/eastmoney/limit_up_pool/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF33" s="6" t="str">
+        <x:v>data/task_workspace/limit_up_pool/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG33" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-045/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH33" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI33" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="89" customHeight="1">
@@ -3329,6 +3850,25 @@
         <x:v>config/providers.yaml#ASTOCK-046
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE34" s="6" t="str">
+        <x:v>data/raw/eastmoney/broken_limit_pool/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF34" s="6" t="str">
+        <x:v>data/task_workspace/broken_limit_pool/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG34" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-046/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH34" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI34" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="89" customHeight="1">
       <x:c r="A35" s="12" t="str">
@@ -3427,6 +3967,25 @@
         <x:v>config/providers.yaml#ASTOCK-047
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE35" s="6" t="str">
+        <x:v>data/raw/eastmoney/limit_down_pool/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF35" s="6" t="str">
+        <x:v>data/task_workspace/limit_down_pool/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG35" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-047/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH35" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI35" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="89" customHeight="1">
       <x:c r="A36" s="12" t="str">
@@ -3525,6 +4084,25 @@
         <x:v>config/providers.yaml#ASTOCK-048
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE36" s="6" t="str">
+        <x:v>data/raw/eastmoney/previous_limit_pool/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF36" s="6" t="str">
+        <x:v>data/task_workspace/previous_limit_pool/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG36" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-048/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH36" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI36" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="89" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -3623,6 +4201,25 @@
       <x:c r="AD37" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-050
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE37" s="6" t="str">
+        <x:v>data/raw/eastmoney/strong_stock_pool/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF37" s="6" t="str">
+        <x:v>data/task_workspace/strong_stock_pool/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG37" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-050/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH37" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI37" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="89" customHeight="1">
@@ -3725,6 +4322,25 @@
         <x:v>config/providers.yaml#ASTOCK-051
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE38" s="6" t="str">
+        <x:v>data/raw/eastmoney/intraday_changes/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF38" s="6" t="str">
+        <x:v>data/task_workspace/intraday_changes/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG38" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-051/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH38" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI38" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="89" customHeight="1">
       <x:c r="A39" s="12" t="str">
@@ -3826,6 +4442,25 @@
         <x:v>config/providers.yaml#ASTOCK-055
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE39" s="6" t="str">
+        <x:v>data/raw/sse/option_risk/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF39" s="6" t="str">
+        <x:v>data/task_workspace/option_risk/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG39" s="6" t="str">
+        <x:v>sources/sse/ASTOCK-055/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH39" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI39" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="116" customHeight="1">
       <x:c r="A40" s="12" t="str">
@@ -3925,6 +4560,25 @@
         <x:v>config/providers.yaml#ASTOCK-061
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE40" s="6" t="str">
+        <x:v>data/raw/mofcom/social_financing/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF40" s="6" t="str">
+        <x:v>data/task_workspace/social_financing/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG40" s="6" t="str">
+        <x:v>sources/mofcom/ASTOCK-061/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH40" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI40" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="89" customHeight="1">
       <x:c r="A41" s="12" t="str">
@@ -4022,6 +4676,25 @@
       <x:c r="AD41" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-062
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE41" s="6" t="str">
+        <x:v>data/raw/eastmoney/pmi/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF41" s="6" t="str">
+        <x:v>data/task_workspace/pmi_history/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG41" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-062/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH41" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI41" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="76" customHeight="1">
@@ -4121,6 +4794,25 @@
       <x:c r="AD42" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-063
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE42" s="6" t="str">
+        <x:v>data/raw/chinabond/yield_curve/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF42" s="6" t="str">
+        <x:v>data/task_workspace/bond_yield_curve/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG42" s="6" t="str">
+        <x:v>sources/chinabond/ASTOCK-063/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH42" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI42" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="103" customHeight="1">
@@ -4224,6 +4916,25 @@
         <x:v>config/providers.yaml#ASTOCK-064
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE43" s="6" t="str">
+        <x:v>data/raw/chinamoney/repo_fixing/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF43" s="6" t="str">
+        <x:v>data/task_workspace/repo_fixing/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG43" s="6" t="str">
+        <x:v>sources/chinamoney/ASTOCK-064/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH43" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI43" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="89" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -4325,6 +5036,25 @@
         <x:v>config/providers.yaml#ASTOCK-065
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE44" s="6" t="str">
+        <x:v>data/raw/eastmoney/lpr/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF44" s="6" t="str">
+        <x:v>data/task_workspace/lpr_history/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG44" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-065/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH44" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI44" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="76" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -4419,6 +5149,25 @@
       <x:c r="AD45" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-066
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE45" s="6" t="str">
+        <x:v>data/raw/wallstreetcn/macro_calendar/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF45" s="6" t="str">
+        <x:v>data/task_workspace/macro_calendar/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG45" s="6" t="str">
+        <x:v>sources/wallstreetcn/ASTOCK-066/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH45" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI45" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="103" customHeight="1">
@@ -4521,6 +5270,25 @@
         <x:v>config/providers.yaml#ASTOCK-067
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE46" s="6" t="str">
+        <x:v>data/raw/csindex/constituents/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF46" s="6" t="str">
+        <x:v>data/task_workspace/index_constituents/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG46" s="6" t="str">
+        <x:v>sources/csindex/ASTOCK-067/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH46" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI46" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="103" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -4622,6 +5390,25 @@
         <x:v>config/providers.yaml#ASTOCK-068
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE47" s="6" t="str">
+        <x:v>data/raw/csindex/weights/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF47" s="6" t="str">
+        <x:v>data/task_workspace/index_weights/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG47" s="6" t="str">
+        <x:v>sources/csindex/ASTOCK-068/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH47" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI47" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="103" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -4725,6 +5512,25 @@
         <x:v>config/providers.yaml#ASTOCK-069
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE48" s="6" t="str">
+        <x:v>data/raw/csindex/index_valuation/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF48" s="6" t="str">
+        <x:v>data/task_workspace/index_valuation/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG48" s="6" t="str">
+        <x:v>sources/csindex/ASTOCK-069/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH48" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI48" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="89" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -4817,6 +5623,25 @@
       <x:c r="AD49" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-070
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE49" s="6" t="str">
+        <x:v>data/raw/sina/trading_calendar/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF49" s="6" t="str">
+        <x:v>data/task_workspace/trading_calendar/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG49" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-070/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH49" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI49" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="103" customHeight="1">
@@ -4920,6 +5745,25 @@
         <x:v>config/providers.yaml#ASTOCK-071
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE50" s="6" t="str">
+        <x:v>data/raw/exchange_composite/futures_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF50" s="6" t="str">
+        <x:v>data/task_workspace/official_futures_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG50" s="6" t="str">
+        <x:v>sources/exchange_composite/ASTOCK-071/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH50" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI50" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="103" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -5022,6 +5866,25 @@
       <x:c r="AD51" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-072
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE51" s="6" t="str">
+        <x:v>data/raw/exchange_composite/options_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF51" s="6" t="str">
+        <x:v>data/task_workspace/official_options_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG51" s="6" t="str">
+        <x:v>sources/exchange_composite/ASTOCK-072/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH51" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI51" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="116" customHeight="1">
@@ -5131,6 +5994,25 @@
         <x:v>config/providers.yaml#ASTOCK-073
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE52" s="6" t="str">
+        <x:v>data/raw/cffex/position_rank/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF52" s="6" t="str">
+        <x:v>data/task_workspace/position_rank/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG52" s="6" t="str">
+        <x:v>sources/cffex/ASTOCK-073/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH52" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI52" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="103" customHeight="1">
       <x:c r="A53" s="12" t="str">
@@ -5233,6 +6115,25 @@
         <x:v>config/providers.yaml#ASTOCK-074
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE53" s="6" t="str">
+        <x:v>data/raw/sina/futures_quote/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF53" s="6" t="str">
+        <x:v>data/task_workspace/futures_quote/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG53" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-074/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH53" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI53" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="103" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -5332,6 +6233,25 @@
       <x:c r="AD54" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-075
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE54" s="6" t="str">
+        <x:v>data/raw/sina/futures_kline/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF54" s="6" t="str">
+        <x:v>data/task_workspace/futures_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG54" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-075/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH54" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI54" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="103" customHeight="1">
@@ -5435,6 +6355,25 @@
         <x:v>config/providers.yaml#ASTOCK-076
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE55" s="6" t="str">
+        <x:v>data/raw/sina/a50_quote/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF55" s="6" t="str">
+        <x:v>data/task_workspace/a50_quote/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG55" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-076/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH55" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI55" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="103" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -5536,6 +6475,25 @@
         <x:v>config/providers.yaml#ASTOCK-077
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE56" s="6" t="str">
+        <x:v>data/raw/sge/spot/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF56" s="6" t="str">
+        <x:v>data/task_workspace/sge_spot/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG56" s="6" t="str">
+        <x:v>sources/sge/ASTOCK-077/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH56" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI56" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="89" customHeight="1">
       <x:c r="A57" s="12" t="str">
@@ -5636,6 +6594,25 @@
         <x:v>config/providers.yaml#ASTOCK-078
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE57" s="6" t="str">
+        <x:v>data/raw/eastmoney/earnings_forecast/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF57" s="6" t="str">
+        <x:v>data/task_workspace/earnings_forecast/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG57" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-078/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH57" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI57" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="89" customHeight="1">
       <x:c r="A58" s="12" t="str">
@@ -5733,6 +6710,25 @@
       <x:c r="AD58" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-079
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE58" s="6" t="str">
+        <x:v>data/raw/eastmoney/institution_survey/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF58" s="6" t="str">
+        <x:v>data/task_workspace/institution_survey/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG58" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-079/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH58" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI58" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="89" customHeight="1">
@@ -5833,6 +6829,25 @@
       <x:c r="AD59" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-080
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE59" s="6" t="str">
+        <x:v>data/raw/eastmoney/holder_trades/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF59" s="6" t="str">
+        <x:v>data/task_workspace/holder_trades/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG59" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-080/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH59" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI59" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="89" customHeight="1">
@@ -5934,6 +6949,25 @@
       <x:c r="AD60" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-081
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE60" s="6" t="str">
+        <x:v>data/raw/eastmoney/buyback/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF60" s="6" t="str">
+        <x:v>data/task_workspace/buyback/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG60" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-081/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH60" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI60" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="103" customHeight="1">
@@ -6037,6 +7071,25 @@
         <x:v>config/providers.yaml#ASTOCK-082
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE61" s="6" t="str">
+        <x:v>data/raw/eastmoney/pledge/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF61" s="6" t="str">
+        <x:v>data/task_workspace/pledge/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG61" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-082/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH61" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI61" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="89" customHeight="1">
       <x:c r="A62" s="12" t="str">
@@ -6137,6 +7190,25 @@
       <x:c r="AD62" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-083
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE62" s="6" t="str">
+        <x:v>data/raw/eastmoney/ipo_calendar/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF62" s="6" t="str">
+        <x:v>data/task_workspace/ipo_calendar/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG62" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-083/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH62" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI62" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="116" customHeight="1">
@@ -6241,6 +7313,25 @@
         <x:v>config/providers.yaml#ASTOCK-084
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE63" s="6" t="str">
+        <x:v>data/raw/eastmoney/convertible_bonds/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF63" s="6" t="str">
+        <x:v>data/task_workspace/convertible_bonds/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG63" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-084/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH63" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI63" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="89" customHeight="1">
       <x:c r="A64" s="12" t="str">
@@ -6340,6 +7431,25 @@
       <x:c r="AD64" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-085
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE64" s="6" t="str">
+        <x:v>data/raw/sina/dragon_tiger_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF64" s="6" t="str">
+        <x:v>data/task_workspace/sina_dragon_tiger_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG64" s="6" t="str">
+        <x:v>sources/sina/ASTOCK-085/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH64" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI64" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="103" customHeight="1">
@@ -6441,6 +7551,25 @@
         <x:v>config/providers.yaml#ASTOCK-087
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE65" s="6" t="str">
+        <x:v>data/raw/eastmoney/dated_announcements/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF65" s="6" t="str">
+        <x:v>data/task_workspace/dated_announcements/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG65" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-087/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH65" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI65" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="62" customHeight="1">
       <x:c r="A66" s="12" t="str">
@@ -6534,6 +7663,25 @@
         <x:v>config/providers.yaml#SDA-BOARD-001
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE66" s="6" t="str">
+        <x:v>data/raw/ths/industry_directory/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF66" s="6" t="str">
+        <x:v>data/task_workspace/industry_directory/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG66" s="6" t="str">
+        <x:v>sources/ths/SDA-BOARD-001/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH66" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI66" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="62" customHeight="1">
       <x:c r="A67" s="12" t="str">
@@ -6627,6 +7775,25 @@
       <x:c r="AD67" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-002
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE67" s="6" t="str">
+        <x:v>data/raw/ths/industry_index_daily/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF67" s="6" t="str">
+        <x:v>data/task_workspace/industry_index_daily/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG67" s="6" t="str">
+        <x:v>sources/ths/SDA-BOARD-002/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH67" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI67" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="89" customHeight="1">
@@ -6722,6 +7889,25 @@
       <x:c r="AD68" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-003
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE68" s="6" t="str">
+        <x:v>data/raw/ths/industry_fund_flow/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF68" s="6" t="str">
+        <x:v>data/task_workspace/board_fund_flow/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG68" s="6" t="str">
+        <x:v>sources/ths/SDA-BOARD-003/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH68" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI68" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="251" customHeight="1">
@@ -6824,6 +8010,25 @@
         <x:v>config/providers.yaml#SDA-BOARD-004
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE69" s="6" t="str">
+        <x:v>data/raw/ths/concept_fund_flow/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF69" s="6" t="str">
+        <x:v>data/task_workspace/board_fund_flow/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG69" s="6" t="str">
+        <x:v>sources/ths/SDA-BOARD-004/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH69" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI69" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="89" customHeight="1">
       <x:c r="A70" s="12" t="str">
@@ -6919,6 +8124,25 @@
         <x:v>config/providers.yaml#SDA-BOARD-005
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE70" s="6" t="str">
+        <x:v>data/raw/baostock/security_snapshot/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF70" s="6" t="str">
+        <x:v>data/task_workspace/security_snapshot/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG70" s="6" t="str">
+        <x:v>sources/baostock/SDA-BOARD-005/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH70" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI70" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="76" customHeight="1">
       <x:c r="A71" s="12" t="str">
@@ -7013,6 +8237,25 @@
       <x:c r="AD71" s="6" t="str">
         <x:v>config/providers.yaml#SDA-BOARD-006
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE71" s="6" t="str">
+        <x:v>data/raw/baostock/industry_membership/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF71" s="6" t="str">
+        <x:v>data/task_workspace/industry_membership/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG71" s="6" t="str">
+        <x:v>sources/baostock/SDA-BOARD-006/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH71" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI71" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="89" customHeight="1">
@@ -7112,6 +8355,25 @@
       <x:c r="AD72" s="6" t="str">
         <x:v>config/providers.yaml#ASTOCK-037-profile
 src/routing/factory.py</x:v>
+      </x:c>
+      <x:c r="AE72" s="6" t="str">
+        <x:v>data/raw/cninfo/company_profile/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF72" s="6" t="str">
+        <x:v>data/task_workspace/company_profile/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG72" s="6" t="str">
+        <x:v>sources/cninfo/ASTOCK-037-profile/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH72" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI72" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="103" customHeight="1">
@@ -7213,11 +8475,30 @@
         <x:v>config/providers.yaml#ASTOCK-037-events
 src/routing/factory.py</x:v>
       </x:c>
+      <x:c r="AE73" s="6" t="str">
+        <x:v>data/raw/eastmoney/company_events/
+&lt;UTC抓取日期&gt;/&lt;批次&gt;/manifest.ndjson
+bodies/&lt;SHA256&gt;.bin</x:v>
+      </x:c>
+      <x:c r="AF73" s="6" t="str">
+        <x:v>data/task_workspace/company_events/scope-&lt;请求范围哈希&gt;/&lt;任务ID&gt;/</x:v>
+      </x:c>
+      <x:c r="AG73" s="6" t="str">
+        <x:v>sources/eastmoney/ASTOCK-037-events/
+normalized.parquet
+normalized.json；parsed/；raw_refs.json</x:v>
+      </x:c>
+      <x:c r="AH73" s="6" t="str">
+        <x:v>data/canonical/ 按数据集及业务分区；本输入仅候选完成，尚未接通正式发布</x:v>
+      </x:c>
+      <x:c r="AI73" s="6" t="str">
+        <x:v>正式发布与元数据状态均成功、文件哈希通过后进入 data/task_archive/；候选和失败任务保留工作区</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d69ae4881b4b29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R231483beaf93473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7287,7 +8568,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.680338136575</x:v>
+        <x:v>46299.7938500463</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -12398,7 +13679,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4702f5b6e1b44f90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f51c708da994543"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12477,7 +13758,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.680338136575</x:v>
+        <x:v>46299.7938500463</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -68968,7 +70249,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R048dd8b2f1d747db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf695ef9eb8fb40b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -69020,7 +70301,7 @@
         <x:v>文档生成时间（UTC）</x:v>
       </x:c>
       <x:c r="B3" s="4" t="n">
-        <x:v>46299.680338136575</x:v>
+        <x:v>46299.7938500463</x:v>
       </x:c>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2"/>
@@ -69478,7 +70759,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2593b588e498429c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0ec0a7fd8ef4dff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>